<commit_message>
filtra y gestiona ofertas y entrega un excel
</commit_message>
<xml_diff>
--- a/vacantes.template.xlsx
+++ b/vacantes.template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vacantes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="vacantes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'vacantes'!$A$1:$O$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'vacantes'!$A$1:$R$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,30 +425,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
     <col width="23" customWidth="1" min="13" max="13"/>
-    <col width="45" customWidth="1" min="14" max="14"/>
-    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>nombre_de_la_vacante</t>
+          <t>titulo</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -463,60 +466,75 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>industria</t>
+          <t>url</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>descripcion</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>ubicacion</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>modalidad</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>salario</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>fecha_publicacion</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>email_contacto</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>industria_detectada</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>fuente_extraccion</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>requiere_intervencion</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>estado_extraccion</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>horas_semana</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>seniority</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>idioma</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>fecha_publicacion</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>email_contacto</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>descripcion</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>url_empresa</t>
         </is>
@@ -540,65 +558,80 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>https://example.com/job</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Buscamos developer con React, TypeScript, Node.js, APIs REST, PostgreSQL, Docker y CI/CD.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Remoto Mexico</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>remoto</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>25000 MXN</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>recruiter@example.com</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>SaaS</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Remoto Mexico</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>remoto</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>25000 MXN</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
         <v>40</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>es</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>https://example.com/job</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>recruiter@example.com</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Buscamos developer con React, TypeScript, Node.js, APIs REST, PostgreSQL, Docker y CI/CD.</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>https://example.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O2"/>
+  <autoFilter ref="A1:R2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>